<commit_message>
remoção de arquivo extra
</commit_message>
<xml_diff>
--- a/templates/contato_setores.xlsx
+++ b/templates/contato_setores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TopFama\Documents\ProjetosDEV\mensageiro_orcamento\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB60E870-F343-4ACE-8925-C596692AE582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B93C07F-E24D-4859-8364-47CC604381A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{027C0934-9CA5-43DA-B860-5C3B087AD038}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
   <si>
     <t>nome</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>COMPRAS</t>
+  </si>
+  <si>
+    <t>5563999514371</t>
   </si>
 </sst>
 </file>
@@ -915,19 +918,25 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1"/>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="1"/>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="1"/>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>

</xml_diff>